<commit_message>
Provide table of full model results
</commit_message>
<xml_diff>
--- a/tables/coverage20_beta_model_results.xlsx
+++ b/tables/coverage20_beta_model_results.xlsx
@@ -11,17 +11,20 @@
     <sheet name="Fixed_effects" sheetId="2" r:id="rId2"/>
     <sheet name="Model_comparison" sheetId="3" r:id="rId3"/>
     <sheet name="EMM_sample_type" sheetId="4" r:id="rId4"/>
-    <sheet name="EMM_temperature" sheetId="5" r:id="rId5"/>
-    <sheet name="Pairwise_sample_type" sheetId="6" r:id="rId6"/>
+    <sheet name="Pairwise_sample_type" sheetId="5" r:id="rId5"/>
+    <sheet name="EMM_temperature" sheetId="6" r:id="rId6"/>
     <sheet name="Pairwise_temperature" sheetId="7" r:id="rId7"/>
-    <sheet name="Random_effects" sheetId="8" r:id="rId8"/>
+    <sheet name="EMM_timepoint" sheetId="8" r:id="rId8"/>
+    <sheet name="Pairwise_timepoint" sheetId="9" r:id="rId9"/>
+    <sheet name="Random_effects" sheetId="10" r:id="rId10"/>
+    <sheet name="Model_diagnostics" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="77">
   <si>
     <t>Term</t>
   </si>
@@ -185,22 +188,73 @@
     <t>21</t>
   </si>
   <si>
+    <t>contrast</t>
+  </si>
+  <si>
+    <t>odds.ratio</t>
+  </si>
+  <si>
+    <t>FTA / RDT</t>
+  </si>
+  <si>
     <t>RT</t>
   </si>
   <si>
     <t>37</t>
   </si>
   <si>
-    <t>contrast</t>
-  </si>
-  <si>
-    <t>odds.ratio</t>
-  </si>
-  <si>
-    <t>FTA / RDT</t>
-  </si>
-  <si>
     <t>RT / 37</t>
+  </si>
+  <si>
+    <t>estimate</t>
+  </si>
+  <si>
+    <t>timepoint1 - timepoint3</t>
+  </si>
+  <si>
+    <t>timepoint1 - timepoint7</t>
+  </si>
+  <si>
+    <t>timepoint1 - timepoint21</t>
+  </si>
+  <si>
+    <t>timepoint3 - timepoint7</t>
+  </si>
+  <si>
+    <t>timepoint3 - timepoint21</t>
+  </si>
+  <si>
+    <t>timepoint7 - timepoint21</t>
+  </si>
+  <si>
+    <t>Random_effect</t>
+  </si>
+  <si>
+    <t>Variance</t>
+  </si>
+  <si>
+    <t>SD</t>
+  </si>
+  <si>
+    <t>sample_id (random intercept)</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Statistic</t>
+  </si>
+  <si>
+    <t>DHARMa uniformity</t>
+  </si>
+  <si>
+    <t>DHARMa dispersion</t>
+  </si>
+  <si>
+    <t>DHARMa outliers</t>
+  </si>
+  <si>
+    <t>DHARMa zero inflation</t>
   </si>
 </sst>
 </file>
@@ -663,6 +717,100 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2">
+        <v>0.291</v>
+      </c>
+      <c r="C2">
+        <v>0.539</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2">
+        <v>0.091</v>
+      </c>
+      <c r="C2">
+        <v>0.524</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3">
+        <v>1.208</v>
+      </c>
+      <c r="C3">
+        <v>0.232</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>0.131</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H14"/>
@@ -1425,18 +1573,18 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>6</v>
+        <v>54</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>12</v>
@@ -1462,258 +1610,130 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B2" t="s">
         <v>48</v>
       </c>
       <c r="C2">
-        <v>0.977</v>
+        <v>1.095</v>
       </c>
       <c r="D2">
-        <v>0.007</v>
+        <v>0.299</v>
       </c>
       <c r="E2" t="s">
         <v>49</v>
       </c>
       <c r="F2">
-        <v>0.958</v>
+        <v>0.641</v>
       </c>
       <c r="G2">
-        <v>0.987</v>
+        <v>1.871</v>
       </c>
       <c r="H2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>11.945</v>
+        <v>0.331</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B3" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C3">
-        <v>0.98</v>
+        <v>1.155</v>
       </c>
       <c r="D3">
-        <v>0.006</v>
+        <v>0.281</v>
       </c>
       <c r="E3" t="s">
         <v>49</v>
       </c>
       <c r="F3">
-        <v>0.964</v>
+        <v>0.717</v>
       </c>
       <c r="G3">
-        <v>0.989</v>
+        <v>1.86</v>
       </c>
       <c r="H3">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>12.413</v>
+        <v>0.593</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>0.553</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C4">
-        <v>0.978</v>
+        <v>1.006</v>
       </c>
       <c r="D4">
-        <v>0.007</v>
+        <v>0.197</v>
       </c>
       <c r="E4" t="s">
         <v>49</v>
       </c>
       <c r="F4">
-        <v>0.96</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="G4">
-        <v>0.988</v>
+        <v>1.477</v>
       </c>
       <c r="H4">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>12.197</v>
+        <v>0.031</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>0.975</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C5">
-        <v>0.966</v>
+        <v>1.251</v>
       </c>
       <c r="D5">
-        <v>0.01</v>
+        <v>0.17</v>
       </c>
       <c r="E5" t="s">
         <v>49</v>
       </c>
       <c r="F5">
-        <v>0.9409999999999999</v>
+        <v>0.959</v>
       </c>
       <c r="G5">
-        <v>0.98</v>
+        <v>1.633</v>
       </c>
       <c r="H5">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>11.528</v>
+        <v>1.649</v>
       </c>
       <c r="J5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="A6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B6" t="s">
-        <v>52</v>
-      </c>
-      <c r="C6">
-        <v>0.963</v>
-      </c>
-      <c r="D6">
-        <v>0.01</v>
-      </c>
-      <c r="E6" t="s">
-        <v>49</v>
-      </c>
-      <c r="F6">
-        <v>0.9370000000000001</v>
-      </c>
-      <c r="G6">
-        <v>0.979</v>
-      </c>
-      <c r="H6">
-        <v>0.5</v>
-      </c>
-      <c r="I6">
-        <v>11.399</v>
-      </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
-      <c r="A7" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" t="s">
-        <v>52</v>
-      </c>
-      <c r="C7">
-        <v>0.9429999999999999</v>
-      </c>
-      <c r="D7">
-        <v>0.015</v>
-      </c>
-      <c r="E7" t="s">
-        <v>49</v>
-      </c>
-      <c r="F7">
-        <v>0.906</v>
-      </c>
-      <c r="G7">
-        <v>0.966</v>
-      </c>
-      <c r="H7">
-        <v>0.5</v>
-      </c>
-      <c r="I7">
-        <v>10.244</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="A8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C8">
-        <v>0.899</v>
-      </c>
-      <c r="D8">
-        <v>0.024</v>
-      </c>
-      <c r="E8" t="s">
-        <v>49</v>
-      </c>
-      <c r="F8">
-        <v>0.842</v>
-      </c>
-      <c r="G8">
-        <v>0.9370000000000001</v>
-      </c>
-      <c r="H8">
-        <v>0.5</v>
-      </c>
-      <c r="I8">
-        <v>8.343</v>
-      </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
-      <c r="A9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B9" t="s">
-        <v>53</v>
-      </c>
-      <c r="C9">
-        <v>0.837</v>
-      </c>
-      <c r="D9">
-        <v>0.035</v>
-      </c>
-      <c r="E9" t="s">
-        <v>49</v>
-      </c>
-      <c r="F9">
-        <v>0.756</v>
-      </c>
-      <c r="G9">
-        <v>0.895</v>
-      </c>
-      <c r="H9">
-        <v>0.5</v>
-      </c>
-      <c r="I9">
-        <v>6.357</v>
-      </c>
-      <c r="J9">
-        <v>0</v>
+        <v>0.099</v>
       </c>
     </row>
   </sheetData>
@@ -1723,18 +1743,18 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>56</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>12</v>
@@ -1760,34 +1780,34 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B2" t="s">
         <v>48</v>
       </c>
       <c r="C2">
-        <v>1.095</v>
+        <v>0.977</v>
       </c>
       <c r="D2">
-        <v>0.299</v>
+        <v>0.007</v>
       </c>
       <c r="E2" t="s">
         <v>49</v>
       </c>
       <c r="F2">
-        <v>0.641</v>
+        <v>0.958</v>
       </c>
       <c r="G2">
-        <v>1.871</v>
+        <v>0.987</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I2">
-        <v>0.331</v>
+        <v>11.945</v>
       </c>
       <c r="J2">
-        <v>0.74</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -1795,63 +1815,63 @@
         <v>58</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C3">
-        <v>1.155</v>
+        <v>0.98</v>
       </c>
       <c r="D3">
-        <v>0.281</v>
+        <v>0.006</v>
       </c>
       <c r="E3" t="s">
         <v>49</v>
       </c>
       <c r="F3">
-        <v>0.717</v>
+        <v>0.964</v>
       </c>
       <c r="G3">
-        <v>1.86</v>
+        <v>0.989</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I3">
-        <v>0.593</v>
+        <v>12.413</v>
       </c>
       <c r="J3">
-        <v>0.553</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C4">
-        <v>1.006</v>
+        <v>0.978</v>
       </c>
       <c r="D4">
-        <v>0.197</v>
+        <v>0.007</v>
       </c>
       <c r="E4" t="s">
         <v>49</v>
       </c>
       <c r="F4">
-        <v>0.6850000000000001</v>
+        <v>0.96</v>
       </c>
       <c r="G4">
-        <v>1.477</v>
+        <v>0.988</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I4">
-        <v>0.031</v>
+        <v>12.197</v>
       </c>
       <c r="J4">
-        <v>0.975</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -1859,31 +1879,159 @@
         <v>58</v>
       </c>
       <c r="B5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5">
+        <v>0.966</v>
+      </c>
+      <c r="D5">
+        <v>0.01</v>
+      </c>
+      <c r="E5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5">
+        <v>0.9409999999999999</v>
+      </c>
+      <c r="G5">
+        <v>0.98</v>
+      </c>
+      <c r="H5">
+        <v>0.5</v>
+      </c>
+      <c r="I5">
+        <v>11.528</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6">
+        <v>0.963</v>
+      </c>
+      <c r="D6">
+        <v>0.01</v>
+      </c>
+      <c r="E6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6">
+        <v>0.9370000000000001</v>
+      </c>
+      <c r="G6">
+        <v>0.979</v>
+      </c>
+      <c r="H6">
+        <v>0.5</v>
+      </c>
+      <c r="I6">
+        <v>11.399</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7">
+        <v>0.9429999999999999</v>
+      </c>
+      <c r="D7">
+        <v>0.015</v>
+      </c>
+      <c r="E7" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7">
+        <v>0.906</v>
+      </c>
+      <c r="G7">
+        <v>0.966</v>
+      </c>
+      <c r="H7">
+        <v>0.5</v>
+      </c>
+      <c r="I7">
+        <v>10.244</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" t="s">
         <v>53</v>
       </c>
-      <c r="C5">
-        <v>1.251</v>
-      </c>
-      <c r="D5">
-        <v>0.17</v>
-      </c>
-      <c r="E5" t="s">
-        <v>49</v>
-      </c>
-      <c r="F5">
-        <v>0.959</v>
-      </c>
-      <c r="G5">
-        <v>1.633</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>1.649</v>
-      </c>
-      <c r="J5">
-        <v>0.099</v>
+      <c r="C8">
+        <v>0.899</v>
+      </c>
+      <c r="D8">
+        <v>0.024</v>
+      </c>
+      <c r="E8" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8">
+        <v>0.842</v>
+      </c>
+      <c r="G8">
+        <v>0.9370000000000001</v>
+      </c>
+      <c r="H8">
+        <v>0.5</v>
+      </c>
+      <c r="I8">
+        <v>8.343</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9">
+        <v>0.837</v>
+      </c>
+      <c r="D9">
+        <v>0.035</v>
+      </c>
+      <c r="E9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F9">
+        <v>0.756</v>
+      </c>
+      <c r="G9">
+        <v>0.895</v>
+      </c>
+      <c r="H9">
+        <v>0.5</v>
+      </c>
+      <c r="I9">
+        <v>6.357</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1898,13 +2046,13 @@
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>12</v>
@@ -2063,17 +2211,682 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1" s="1" customFormat="1">
+    <row r="1" spans="1:10" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
-      <c r="A2">
-        <v>0.291016955658019</v>
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2">
+        <v>0.98</v>
+      </c>
+      <c r="D2">
+        <v>0.006</v>
+      </c>
+      <c r="E2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2">
+        <v>0.963</v>
+      </c>
+      <c r="G2">
+        <v>0.989</v>
+      </c>
+      <c r="H2">
+        <v>0.5</v>
+      </c>
+      <c r="I2">
+        <v>12.155</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3">
+        <v>0.974</v>
+      </c>
+      <c r="D3">
+        <v>0.008</v>
+      </c>
+      <c r="E3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3">
+        <v>0.954</v>
+      </c>
+      <c r="G3">
+        <v>0.986</v>
+      </c>
+      <c r="H3">
+        <v>0.5</v>
+      </c>
+      <c r="I3">
+        <v>11.931</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4">
+        <v>0.954</v>
+      </c>
+      <c r="D4">
+        <v>0.012</v>
+      </c>
+      <c r="E4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4">
+        <v>0.923</v>
+      </c>
+      <c r="G4">
+        <v>0.973</v>
+      </c>
+      <c r="H4">
+        <v>0.5</v>
+      </c>
+      <c r="I4">
+        <v>10.877</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5">
+        <v>0.883</v>
+      </c>
+      <c r="D5">
+        <v>0.027</v>
+      </c>
+      <c r="E5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5">
+        <v>0.819</v>
+      </c>
+      <c r="G5">
+        <v>0.927</v>
+      </c>
+      <c r="H5">
+        <v>0.5</v>
+      </c>
+      <c r="I5">
+        <v>7.723</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6">
+        <v>0.978</v>
+      </c>
+      <c r="D6">
+        <v>0.007</v>
+      </c>
+      <c r="E6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6">
+        <v>0.96</v>
+      </c>
+      <c r="G6">
+        <v>0.988</v>
+      </c>
+      <c r="H6">
+        <v>0.5</v>
+      </c>
+      <c r="I6">
+        <v>12.202</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7">
+        <v>0.971</v>
+      </c>
+      <c r="D7">
+        <v>0.008</v>
+      </c>
+      <c r="E7" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7">
+        <v>0.949</v>
+      </c>
+      <c r="G7">
+        <v>0.983</v>
+      </c>
+      <c r="H7">
+        <v>0.5</v>
+      </c>
+      <c r="I7">
+        <v>11.863</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8">
+        <v>0.954</v>
+      </c>
+      <c r="D8">
+        <v>0.012</v>
+      </c>
+      <c r="E8" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8">
+        <v>0.923</v>
+      </c>
+      <c r="G8">
+        <v>0.973</v>
+      </c>
+      <c r="H8">
+        <v>0.5</v>
+      </c>
+      <c r="I8">
+        <v>10.817</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9">
+        <v>0.858</v>
+      </c>
+      <c r="D9">
+        <v>0.031</v>
+      </c>
+      <c r="E9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F9">
+        <v>0.785</v>
+      </c>
+      <c r="G9">
+        <v>0.909</v>
+      </c>
+      <c r="H9">
+        <v>0.5</v>
+      </c>
+      <c r="I9">
+        <v>6.983</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:9" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2">
+        <v>0.233</v>
+      </c>
+      <c r="D2">
+        <v>0.268</v>
+      </c>
+      <c r="E2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2">
+        <v>-0.457</v>
+      </c>
+      <c r="G2">
+        <v>0.922</v>
+      </c>
+      <c r="H2">
+        <v>0.867</v>
+      </c>
+      <c r="I2">
+        <v>0.822</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3">
+        <v>0.84</v>
+      </c>
+      <c r="D3">
+        <v>0.246</v>
+      </c>
+      <c r="E3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3">
+        <v>0.209</v>
+      </c>
+      <c r="G3">
+        <v>1.472</v>
+      </c>
+      <c r="H3">
+        <v>3.418</v>
+      </c>
+      <c r="I3">
+        <v>0.004</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4">
+        <v>1.847</v>
+      </c>
+      <c r="D4">
+        <v>0.226</v>
+      </c>
+      <c r="E4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4">
+        <v>1.267</v>
+      </c>
+      <c r="G4">
+        <v>2.428</v>
+      </c>
+      <c r="H4">
+        <v>8.177</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5">
+        <v>0.608</v>
+      </c>
+      <c r="D5">
+        <v>0.229</v>
+      </c>
+      <c r="E5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5">
+        <v>0.02</v>
+      </c>
+      <c r="G5">
+        <v>1.195</v>
+      </c>
+      <c r="H5">
+        <v>2.658</v>
+      </c>
+      <c r="I5">
+        <v>0.039</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6">
+        <v>1.615</v>
+      </c>
+      <c r="D6">
+        <v>0.207</v>
+      </c>
+      <c r="E6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6">
+        <v>1.082</v>
+      </c>
+      <c r="G6">
+        <v>2.147</v>
+      </c>
+      <c r="H6">
+        <v>7.786</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7">
+        <v>1.007</v>
+      </c>
+      <c r="D7">
+        <v>0.17</v>
+      </c>
+      <c r="E7" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7">
+        <v>0.569</v>
+      </c>
+      <c r="G7">
+        <v>1.445</v>
+      </c>
+      <c r="H7">
+        <v>5.912</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8">
+        <v>0.286</v>
+      </c>
+      <c r="D8">
+        <v>0.25</v>
+      </c>
+      <c r="E8" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8">
+        <v>-0.357</v>
+      </c>
+      <c r="G8">
+        <v>0.929</v>
+      </c>
+      <c r="H8">
+        <v>1.143</v>
+      </c>
+      <c r="I8">
+        <v>0.663</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9">
+        <v>0.756</v>
+      </c>
+      <c r="D9">
+        <v>0.236</v>
+      </c>
+      <c r="E9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F9">
+        <v>0.149</v>
+      </c>
+      <c r="G9">
+        <v>1.362</v>
+      </c>
+      <c r="H9">
+        <v>3.2</v>
+      </c>
+      <c r="I9">
+        <v>0.008</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10">
+        <v>1.981</v>
+      </c>
+      <c r="D10">
+        <v>0.212</v>
+      </c>
+      <c r="E10" t="s">
+        <v>49</v>
+      </c>
+      <c r="F10">
+        <v>1.435</v>
+      </c>
+      <c r="G10">
+        <v>2.526</v>
+      </c>
+      <c r="H10">
+        <v>9.327</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11">
+        <v>0.47</v>
+      </c>
+      <c r="D11">
+        <v>0.217</v>
+      </c>
+      <c r="E11" t="s">
+        <v>49</v>
+      </c>
+      <c r="F11">
+        <v>-0.08799999999999999</v>
+      </c>
+      <c r="G11">
+        <v>1.027</v>
+      </c>
+      <c r="H11">
+        <v>2.164</v>
+      </c>
+      <c r="I11">
+        <v>0.133</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12">
+        <v>1.695</v>
+      </c>
+      <c r="D12">
+        <v>0.19</v>
+      </c>
+      <c r="E12" t="s">
+        <v>49</v>
+      </c>
+      <c r="F12">
+        <v>1.206</v>
+      </c>
+      <c r="G12">
+        <v>2.183</v>
+      </c>
+      <c r="H12">
+        <v>8.907999999999999</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13">
+        <v>1.225</v>
+      </c>
+      <c r="D13">
+        <v>0.167</v>
+      </c>
+      <c r="E13" t="s">
+        <v>49</v>
+      </c>
+      <c r="F13">
+        <v>0.797</v>
+      </c>
+      <c r="G13">
+        <v>1.653</v>
+      </c>
+      <c r="H13">
+        <v>7.352</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>